<commit_message>
Etapa 1: compra de trompo, vibradora y encofrado fenólico en costos internos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JDAvj83gCUU9yQbmQvUtv6
</commit_message>
<xml_diff>
--- a/metrados/Etapa1_Presupuesto_Informal_INTERNO.xlsx
+++ b/metrados/Etapa1_Presupuesto_Informal_INTERNO.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="391">
   <si>
     <t xml:space="preserve">COTIZACIÓN ETAPA 1 - VIVIENDA UNIFAMILIAR, CHORRILLOS</t>
   </si>
@@ -691,13 +691,52 @@
     <t xml:space="preserve">Alquiler vibrador</t>
   </si>
   <si>
-    <t xml:space="preserve">encof</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alquiler / reposición de encofrado (tablas, puntales, fenólico)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tu Excel 2,000; +500 por VE sobre zapata</t>
+    <t xml:space="preserve">trompo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trompo (mezcladora) - compra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vibc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vibradora de concreto - compra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Triplay fenólico film 18 mm 1.22×2.44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sodimac: S/ 85-107 por 10 o más unidades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nfen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cantidad de planchas fenólicas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">83 m² de VE+VC a la vez, 3 piezas de 0.70×1.22 por plancha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listones, estacas, tensores y tirafondos para encofrado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: ~60 listones 2"x3"x10' + accesorios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">resid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor que te queda en equipos y encofrado al terminar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trompo/vibradora ~75%, fenólico tras 4-5 usos ~30%</t>
   </si>
   <si>
     <t xml:space="preserve">MATERIALES - ETAPA 1 (cantidades por despiece real de varillas)</t>
@@ -1087,13 +1126,22 @@
     <t xml:space="preserve">Confirmar si está incluido</t>
   </si>
   <si>
-    <t xml:space="preserve">Alquiler / reposición de encofrado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mezcladora (4 días) y vibrador (2 días)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solados, ciclópeo, sobrecimiento, solera, mortero; vibrado de premezclado</t>
+    <t xml:space="preserve">Compra trompo (mezcladora)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Queda para otras obras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra vibradora de concreto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra encofrado: fenólico 18 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32 planchas: VE+VC (83 m²) van en un solo vaciado; luego se reusan en columnas, sobrecimiento y cerco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compra encofrado: listones 2"x3"x10', estacas, tensores</t>
   </si>
   <si>
     <t xml:space="preserve">SCTR + EPP (casco, botas, guantes, lentes)</t>
@@ -1111,7 +1159,7 @@
     <t xml:space="preserve">~10 semanas</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL DE MIS COSTOS</t>
+    <t xml:space="preserve">TOTAL DE MIS COSTOS (salida de caja)</t>
   </si>
   <si>
     <t xml:space="preserve">COBRO DE MANO DE OBRA AL CLIENTE</t>
@@ -1120,16 +1168,28 @@
     <t xml:space="preserve">Hoja Mano de obra (redondeado)</t>
   </si>
   <si>
-    <t xml:space="preserve">MI GANANCIA (incluye pago por mi trabajo y dirección)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ganancia por semana</t>
+    <t xml:space="preserve">MI GANANCIA EN EFECTIVO (cobro - salida de caja)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lo que te queda en el bolsillo al terminar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor de equipos y encofrado que te quedan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los puedes usar en la siguiente obra o vender</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MI GANANCIA REAL (efectivo + equipos que te quedan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ganancia real por semana</t>
   </si>
   <si>
     <t xml:space="preserve">Compárala con lo que ganarías como operario (~S/ 780/semana)</t>
   </si>
   <si>
-    <t xml:space="preserve">Margen sobre lo cobrado</t>
+    <t xml:space="preserve">Margen real sobre lo cobrado</t>
   </si>
   <si>
     <t xml:space="preserve">SENSIBILIDAD - si la obra se demora más</t>
@@ -1138,7 +1198,7 @@
     <t xml:space="preserve">Días hábiles reales</t>
   </si>
   <si>
-    <t xml:space="preserve">Mi ganancia (S/)</t>
+    <t xml:space="preserve">Mi ganancia real (S/)</t>
   </si>
 </sst>
 </file>
@@ -2791,7 +2851,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -3363,13 +3423,98 @@
         <v>222</v>
       </c>
       <c r="C36" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D36" s="15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D37" s="15" t="n">
+        <v>400</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="D38" s="15" t="n">
+        <v>95</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D39" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="C40" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="D36" s="15" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>223</v>
+      <c r="D40" s="15" t="n">
+        <v>900</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D41" s="15" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -3401,40 +3546,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="B5" s="14"/>
       <c r="C5" s="14"/>
@@ -3448,7 +3593,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>49</v>
@@ -3465,7 +3610,7 @@
         <v>12800</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3473,7 +3618,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>49</v>
@@ -3496,7 +3641,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>49</v>
@@ -3513,7 +3658,7 @@
         <v>3040</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3521,7 +3666,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>49</v>
@@ -3538,12 +3683,12 @@
         <v>760</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>240</v>
+        <v>253</v>
       </c>
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
@@ -3557,7 +3702,7 @@
         <v>5</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>148</v>
@@ -3574,7 +3719,7 @@
         <v>1687.4</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>242</v>
+        <v>255</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3582,7 +3727,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>49</v>
@@ -3599,7 +3744,7 @@
         <v>576</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3607,7 +3752,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>49</v>
@@ -3624,7 +3769,7 @@
         <v>175.5</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3632,7 +3777,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>49</v>
@@ -3655,7 +3800,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>248</v>
+        <v>261</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>49</v>
@@ -3678,7 +3823,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>249</v>
+        <v>262</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>49</v>
@@ -3698,7 +3843,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>250</v>
+        <v>263</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
@@ -3729,7 +3874,7 @@
         <v>5761.44</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>251</v>
+        <v>264</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3754,7 +3899,7 @@
         <v>11262.87</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>252</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3779,7 +3924,7 @@
         <v>6436.84</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>253</v>
+        <v>266</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3804,7 +3949,7 @@
         <v>2688.04</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>254</v>
+        <v>267</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3829,7 +3974,7 @@
         <v>119.4</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>255</v>
+        <v>268</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3837,7 +3982,7 @@
         <v>16</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>256</v>
+        <v>269</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>174</v>
@@ -3854,12 +3999,12 @@
         <v>699.8</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
       <c r="B24" s="14"/>
       <c r="C24" s="14"/>
@@ -3873,7 +4018,7 @@
         <v>17</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>259</v>
+        <v>272</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>109</v>
@@ -3890,7 +4035,7 @@
         <v>364</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>260</v>
+        <v>273</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3898,7 +4043,7 @@
         <v>18</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>261</v>
+        <v>274</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>109</v>
@@ -3915,7 +4060,7 @@
         <v>262.5</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3923,7 +4068,7 @@
         <v>19</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>113</v>
@@ -3940,7 +4085,7 @@
         <v>4058.4</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>264</v>
+        <v>277</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3948,7 +4093,7 @@
         <v>20</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>265</v>
+        <v>278</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>185</v>
@@ -3965,7 +4110,7 @@
         <v>165</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>266</v>
+        <v>279</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3973,7 +4118,7 @@
         <v>21</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>267</v>
+        <v>280</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>185</v>
@@ -3990,7 +4135,7 @@
         <v>80</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>268</v>
+        <v>281</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3998,7 +4143,7 @@
         <v>22</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>269</v>
+        <v>282</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>113</v>
@@ -4015,7 +4160,7 @@
         <v>120</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>270</v>
+        <v>283</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4023,7 +4168,7 @@
         <v>23</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>192</v>
@@ -4080,7 +4225,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>272</v>
+        <v>285</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4088,7 +4233,7 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -4097,16 +4242,16 @@
         <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>273</v>
+        <v>286</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4114,7 +4259,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>274</v>
+        <v>287</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>195</v>
@@ -4131,7 +4276,7 @@
         <v>2300</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>275</v>
+        <v>288</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4139,7 +4284,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>276</v>
+        <v>289</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>199</v>
@@ -4156,7 +4301,7 @@
         <v>1040</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>277</v>
+        <v>290</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4181,7 +4326,7 @@
         <v>375</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>278</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4189,7 +4334,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>279</v>
+        <v>292</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>192</v>
@@ -4212,7 +4357,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>280</v>
+        <v>293</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>127</v>
@@ -4234,7 +4379,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>127</v>
@@ -4250,7 +4395,7 @@
         <v>300</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>282</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4294,12 +4439,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>283</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>284</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4313,23 +4458,23 @@
         <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>285</v>
+        <v>298</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3" t="s">
-        <v>287</v>
+        <v>300</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>288</v>
+        <v>301</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>273</v>
+        <v>286</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4397,7 +4542,7 @@
         <v>47</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>289</v>
+        <v>302</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>49</v>
@@ -4414,13 +4559,13 @@
         <v>3564.8</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>290</v>
+        <v>303</v>
       </c>
       <c r="I7" s="26" t="n">
         <v>0</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>291</v>
+        <v>304</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4428,7 +4573,7 @@
         <v>51</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>292</v>
+        <v>305</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>42</v>
@@ -4451,7 +4596,7 @@
         <v>3.008</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>293</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4459,7 +4604,7 @@
         <v>54</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>49</v>
@@ -4489,7 +4634,7 @@
         <v>57</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>49</v>
@@ -4513,7 +4658,7 @@
         <v>7.6375</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>296</v>
+        <v>309</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4521,7 +4666,7 @@
         <v>64</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>297</v>
+        <v>310</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>42</v>
@@ -4551,7 +4696,7 @@
         <v>67</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>298</v>
+        <v>311</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>49</v>
@@ -4581,7 +4726,7 @@
         <v>70</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>299</v>
+        <v>312</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>49</v>
@@ -4611,7 +4756,7 @@
         <v>73</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>300</v>
+        <v>313</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>42</v>
@@ -4638,10 +4783,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>301</v>
+        <v>314</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>109</v>
@@ -4667,10 +4812,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>109</v>
@@ -4699,7 +4844,7 @@
         <v>83</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>42</v>
@@ -4722,7 +4867,7 @@
         <v>6.90833333333333</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>306</v>
+        <v>319</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4730,7 +4875,7 @@
         <v>86</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>307</v>
+        <v>320</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>42</v>
@@ -4760,7 +4905,7 @@
         <v>77</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>308</v>
+        <v>321</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>49</v>
@@ -4783,15 +4928,15 @@
         <v>1</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>309</v>
+        <v>322</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>310</v>
+        <v>323</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>311</v>
+        <v>324</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>109</v>
@@ -4814,7 +4959,7 @@
         <v>13.23</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>312</v>
+        <v>325</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4822,7 +4967,7 @@
         <v>98</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>313</v>
+        <v>326</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>42</v>
@@ -4852,7 +4997,7 @@
         <v>95</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>314</v>
+        <v>327</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>49</v>
@@ -4875,15 +5020,15 @@
         <v>1</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>315</v>
+        <v>328</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>316</v>
+        <v>329</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>317</v>
+        <v>330</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>109</v>
@@ -4912,7 +5057,7 @@
         <v>104</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>318</v>
+        <v>331</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>42</v>
@@ -4939,10 +5084,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>319</v>
+        <v>332</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>320</v>
+        <v>333</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>49</v>
@@ -4971,7 +5116,7 @@
         <v>111</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>321</v>
+        <v>334</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>113</v>
@@ -5001,7 +5146,7 @@
         <v>115</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>42</v>
@@ -5031,7 +5176,7 @@
         <v>117</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>323</v>
+        <v>336</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>42</v>
@@ -5091,7 +5236,7 @@
         <v>125</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>324</v>
+        <v>337</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>199</v>
@@ -5114,15 +5259,15 @@
         <v>1</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>325</v>
+        <v>338</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>326</v>
+        <v>339</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>327</v>
+        <v>340</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>127</v>
@@ -5148,7 +5293,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="4" t="s">
-        <v>328</v>
+        <v>341</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>127</v>
@@ -5173,7 +5318,7 @@
         <v>30357.8</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="I33" s="27" t="n">
         <f aca="false">SUM(I5:I31)</f>
@@ -5182,7 +5327,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E34" s="28" t="s">
-        <v>330</v>
+        <v>343</v>
       </c>
       <c r="F34" s="29" t="n">
         <f aca="false">CEILING(F33,500)</f>
@@ -5205,7 +5350,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -5215,12 +5360,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>331</v>
+        <v>344</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>332</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5228,68 +5373,68 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>333</v>
+        <v>346</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>334</v>
+        <v>347</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>335</v>
+        <v>348</v>
       </c>
       <c r="B5" s="26" t="n">
         <f aca="false">'Mano de obra'!$I$33</f>
         <v>79.0450714285714</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>336</v>
+        <v>349</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>337</v>
+        <v>350</v>
       </c>
       <c r="B6" s="30" t="n">
         <v>1.35</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>338</v>
+        <v>351</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>339</v>
+        <v>352</v>
       </c>
       <c r="B7" s="31" t="n">
         <v>0.1</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>340</v>
+        <v>353</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>341</v>
+        <v>354</v>
       </c>
       <c r="B8" s="32" t="n">
         <f aca="false">ROUNDUP(B5/B6*(1+B7),0)</f>
         <v>65</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>342</v>
+        <v>355</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>343</v>
+        <v>356</v>
       </c>
       <c r="B9" s="26" t="n">
         <f aca="false">B8/6</f>
         <v>10.8333333333333</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>344</v>
+        <v>357</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5298,13 +5443,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>345</v>
+        <v>358</v>
       </c>
       <c r="C11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>346</v>
+        <v>359</v>
       </c>
       <c r="B12" s="32" t="n">
         <f aca="false">B8*Precios!$D$32</f>
@@ -5314,7 +5459,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>347</v>
+        <v>360</v>
       </c>
       <c r="B13" s="32" t="n">
         <f aca="false">B8*Precios!$D$33</f>
@@ -5324,26 +5469,26 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>348</v>
+        <v>361</v>
       </c>
       <c r="B14" s="32" t="n">
         <f aca="false">6*Precios!$D$33</f>
         <v>480</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>349</v>
+        <v>362</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>350</v>
+        <v>363</v>
       </c>
       <c r="B15" s="32" t="n">
         <f aca="false">13*Precios!$D$30</f>
         <v>1950</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>351</v>
+        <v>364</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5355,185 +5500,233 @@
         <v>300</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>352</v>
+        <v>365</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>353</v>
+        <v>366</v>
       </c>
       <c r="B17" s="32" t="n">
         <f aca="false">Precios!$D$36</f>
-        <v>2500</v>
-      </c>
-      <c r="C17" s="4"/>
+        <v>1000</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>354</v>
+        <v>368</v>
       </c>
       <c r="B18" s="32" t="n">
-        <f aca="false">4*Precios!$D$34+2*Precios!$D$35</f>
-        <v>560</v>
+        <f aca="false">Precios!$D$37</f>
+        <v>400</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>355</v>
+        <v>367</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="B19" s="33" t="n">
-        <v>600</v>
+        <v>369</v>
+      </c>
+      <c r="B19" s="32" t="n">
+        <f aca="false">Precios!$D$39*Precios!$D$38</f>
+        <v>3040</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>357</v>
+        <v>370</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>358</v>
-      </c>
-      <c r="B20" s="33" t="n">
-        <v>400</v>
+        <v>371</v>
+      </c>
+      <c r="B20" s="32" t="n">
+        <f aca="false">Precios!$D$40</f>
+        <v>900</v>
       </c>
       <c r="C20" s="4"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>359</v>
+        <v>372</v>
       </c>
       <c r="B21" s="33" t="n">
         <v>600</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>360</v>
+        <v>373</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>361</v>
-      </c>
-      <c r="B22" s="34" t="n">
-        <f aca="false">SUM(B12:B21)</f>
-        <v>21040</v>
+      <c r="A22" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="B22" s="33" t="n">
+        <v>400</v>
       </c>
       <c r="C22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4"/>
-      <c r="C23" s="4"/>
+      <c r="A23" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="B23" s="33" t="n">
+        <v>600</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>376</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
       <c r="B24" s="34" t="n">
+        <f aca="false">SUM(B12:B23)</f>
+        <v>23320</v>
+      </c>
+      <c r="C24" s="4"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4"/>
+      <c r="C25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="7" t="s">
+        <v>378</v>
+      </c>
+      <c r="B26" s="34" t="n">
         <f aca="false">'Mano de obra'!$F$34</f>
         <v>30500</v>
       </c>
-      <c r="C24" s="4" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="s">
-        <v>364</v>
-      </c>
-      <c r="B25" s="34" t="n">
-        <f aca="false">B24-B22</f>
-        <v>9460</v>
-      </c>
-      <c r="C25" s="4"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
-        <v>365</v>
-      </c>
-      <c r="B26" s="32" t="n">
-        <f aca="false">B25/B9</f>
-        <v>873.230769230769</v>
-      </c>
       <c r="C26" s="4" t="s">
-        <v>366</v>
+        <v>379</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
-        <v>367</v>
-      </c>
-      <c r="B27" s="6" t="n">
-        <f aca="false">B25/B24</f>
-        <v>0.31016393442623</v>
-      </c>
-      <c r="C27" s="4"/>
+      <c r="A27" s="7" t="s">
+        <v>380</v>
+      </c>
+      <c r="B27" s="34" t="n">
+        <f aca="false">B26-B24</f>
+        <v>7180</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="B28" s="32" t="n">
+        <f aca="false">(B17+B18+B19+B20)*Precios!$D$41</f>
+        <v>2403</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>383</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="9" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
-        <v>369</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>370</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>273</v>
+      <c r="A29" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="B29" s="34" t="n">
+        <f aca="false">B27+B28</f>
+        <v>9583</v>
+      </c>
+      <c r="C29" s="4"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="B30" s="32" t="n">
+        <f aca="false">B29/B9</f>
+        <v>884.584615384615</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>386</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="25" t="n">
-        <v>50</v>
-      </c>
-      <c r="B31" s="32" t="n">
-        <f aca="false">B24-(B22-B12-B13+50*(Precios!$D$32+Precios!$D$33))</f>
-        <v>12610</v>
+      <c r="A31" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="B31" s="6" t="n">
+        <f aca="false">B29/B26</f>
+        <v>0.314196721311475</v>
       </c>
       <c r="C31" s="4"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="25" t="n">
-        <v>60</v>
-      </c>
-      <c r="B32" s="32" t="n">
-        <f aca="false">B24-(B22-B12-B13+60*(Precios!$D$32+Precios!$D$33))</f>
-        <v>10510</v>
-      </c>
-      <c r="C32" s="4"/>
-    </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="25" t="n">
-        <v>70</v>
-      </c>
-      <c r="B33" s="32" t="n">
-        <f aca="false">B24-(B22-B12-B13+70*(Precios!$D$32+Precios!$D$33))</f>
-        <v>8410</v>
-      </c>
-      <c r="C33" s="4"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="25" t="n">
-        <v>80</v>
-      </c>
-      <c r="B34" s="32" t="n">
-        <f aca="false">B24-(B22-B12-B13+80*(Precios!$D$32+Precios!$D$33))</f>
-        <v>6310</v>
-      </c>
-      <c r="C34" s="4"/>
+      <c r="A33" s="9" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>286</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="25" t="n">
+        <v>50</v>
+      </c>
+      <c r="B35" s="32" t="n">
+        <f aca="false">B29-(50-B8)*(Precios!$D$32+Precios!$D$33)</f>
+        <v>12733</v>
+      </c>
+      <c r="C35" s="4"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="25" t="n">
+        <v>60</v>
+      </c>
+      <c r="B36" s="32" t="n">
+        <f aca="false">B29-(60-B8)*(Precios!$D$32+Precios!$D$33)</f>
+        <v>10633</v>
+      </c>
+      <c r="C36" s="4"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="25" t="n">
+        <v>70</v>
+      </c>
+      <c r="B37" s="32" t="n">
+        <f aca="false">B29-(70-B8)*(Precios!$D$32+Precios!$D$33)</f>
+        <v>8533</v>
+      </c>
+      <c r="C37" s="4"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="25" t="n">
+        <v>80</v>
+      </c>
+      <c r="B38" s="32" t="n">
+        <f aca="false">B29-(80-B8)*(Precios!$D$32+Precios!$D$33)</f>
+        <v>6433</v>
+      </c>
+      <c r="C38" s="4"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="25" t="n">
         <v>90</v>
       </c>
-      <c r="B35" s="32" t="n">
-        <f aca="false">B24-(B22-B12-B13+90*(Precios!$D$32+Precios!$D$33))</f>
-        <v>4210</v>
-      </c>
-      <c r="C35" s="4"/>
+      <c r="B39" s="32" t="n">
+        <f aca="false">B29-(90-B8)*(Precios!$D$32+Precios!$D$33)</f>
+        <v>4333</v>
+      </c>
+      <c r="C39" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Etapa 1: MO a S/ 36,000 y corrección de sobrecimiento, relleno y premezclado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JDAvj83gCUU9yQbmQvUtv6
</commit_message>
<xml_diff>
--- a/metrados/Etapa1_Presupuesto_Informal_INTERNO.xlsx
+++ b/metrados/Etapa1_Presupuesto_Informal_INTERNO.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="395">
   <si>
     <t xml:space="preserve">COTIZACIÓN ETAPA 1 - VIVIENDA UNIFAMILIAR, CHORRILLOS</t>
   </si>
@@ -205,7 +205,7 @@
     <t xml:space="preserve">Relleno compactado con material propio hasta -0.20</t>
   </si>
   <si>
-    <t xml:space="preserve">Vivienda: 111.4 excav. - 43.1 enterrado - 14.5 (capa superior 0.20) = 53.8; cerco 7.3. E-10 79.4 NO CABE en la excavación</t>
+    <t xml:space="preserve">Vivienda: 111.4 excav. - 44.9 enterrado (incl. sobrecimiento bajo -0.20) - 14.5 (capa superior 0.20) = 52.0; cerco 7.3. E-10 79.4 NO CABE en la excavación</t>
   </si>
   <si>
     <t xml:space="preserve">02.05</t>
@@ -214,7 +214,7 @@
     <t xml:space="preserve">Eliminación de material excedente (esponj. 25%)</t>
   </si>
   <si>
-    <t xml:space="preserve">(124.7 - 61.1) × 1.25. E-10 sale bajo porque su relleno está inflado</t>
+    <t xml:space="preserve">(124.7 - 59.3) × 1.25. E-10 sale bajo porque su relleno está inflado</t>
   </si>
   <si>
     <t xml:space="preserve">03  CONCRETO SIMPLE</t>
@@ -241,10 +241,10 @@
     <t xml:space="preserve">03.03</t>
   </si>
   <si>
-    <t xml:space="preserve">Sobrecimiento 1:8 + 25% PM 0.15×0.40 (perímetro + cerco)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(31.7 + 11.8) × 0.15 × 0.40</t>
+    <t xml:space="preserve">Sobrecimiento 1:8 + 25% PM 0.15 de ancho (perímetro + cerco)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Debe arrancar desde la viga, no desde -0.20: sobre VE (top -0.30) h = 0.50 → 20.98 m; sobre VC de ejes A y C (top -1.10) h ≈ 1.25 → 10.72 m; cerco h = 0.40 → 11.78 m</t>
   </si>
   <si>
     <t xml:space="preserve">03.04</t>
@@ -253,7 +253,7 @@
     <t xml:space="preserve">Encofrado de sobrecimiento (2 caras)</t>
   </si>
   <si>
-    <t xml:space="preserve">43.5 × 0.40 × 2</t>
+    <t xml:space="preserve">2 × (0.50 × 20.98 + 1.25 × 10.72 + 0.40 × 11.78)</t>
   </si>
   <si>
     <t xml:space="preserve">04  CONCRETO ARMADO f'c 210</t>
@@ -265,7 +265,7 @@
     <t xml:space="preserve">Zapatas Z-1 a Z-5 (vaciado contra terreno)</t>
   </si>
   <si>
-    <t xml:space="preserve">Cuadro E-01</t>
+    <t xml:space="preserve">Cuadro E-01. OJO: la excavación lleva 0.10 de sobreancho; si se vacía contra terreno, ese hueco se llena de concreto (+3.8 m³). Perfilar a la medida exacta los 0.50 inferiores</t>
   </si>
   <si>
     <t xml:space="preserve">04.02</t>
@@ -430,6 +430,9 @@
     <t xml:space="preserve">Acero de columnas 1er piso: 2,646 kg (E-10) verificado (barras Ø5/8" de 6.00 m de arranque + estribos Ø1/2" 1,342 kg + montaje 3/8" 38 kg).</t>
   </si>
   <si>
+    <t xml:space="preserve">Diferencias menores a favor (no se cambian): zanjas de VE medidas sin descontar el sobreancho de los pozos (~2.5 m³ de más); encofrado de columnas sin descontar las caras donde llega la VE (~6.7 m²).</t>
+  </si>
+  <si>
     <t xml:space="preserve">PRECIOS DE MATERIALES Y SERVICIOS - Lima, octubre 2026 (con IGV)</t>
   </si>
   <si>
@@ -769,7 +772,7 @@
     <t xml:space="preserve">Premezclado f'c 210 - vaciado 1: zapatas + VE + VC + ZC + VA cerco</t>
   </si>
   <si>
-    <t xml:space="preserve">(23.39 + 11.65 + 0.66 + 1.36 + 1.18) × 1.04 = 39.8 → pedir 40.0</t>
+    <t xml:space="preserve">(23.39 + 11.65 + 0.66 + 1.36 + 1.18) × 1.04 = 39.8 + 2.0 por sobreexcavación de la retro → 42.0</t>
   </si>
   <si>
     <t xml:space="preserve">Bomba - vaciado 1</t>
@@ -793,13 +796,13 @@
     <t xml:space="preserve">Cemento (solado, ciclópeo, sobrecimiento, solera, mortero)</t>
   </si>
   <si>
-    <t xml:space="preserve">Solado 17 + ciclópeo 7 + sobrecim. 11 + solera 4 + mortero 22</t>
+    <t xml:space="preserve">Solado 17 + ciclópeo 7 + sobrecim. 17 + solera 4 + mortero 22</t>
   </si>
   <si>
     <t xml:space="preserve">Hormigón (solado, ciclópeo, sobrecimiento)</t>
   </si>
   <si>
-    <t xml:space="preserve">5.4 + 1.9 + 2.3</t>
+    <t xml:space="preserve">5.4 + 1.9 + 3.7</t>
   </si>
   <si>
     <t xml:space="preserve">Arena gruesa (solera + mortero de muros)</t>
@@ -847,13 +850,13 @@
     <t xml:space="preserve">Alambre N°8 (encofrado)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.25 kg/m² × 224 m²</t>
+    <t xml:space="preserve">0.25 kg/m² × 246 m²</t>
   </si>
   <si>
     <t xml:space="preserve">Clavos</t>
   </si>
   <si>
-    <t xml:space="preserve">0.15 kg/m² × 224 m²</t>
+    <t xml:space="preserve">0.15 kg/m² × 246 m²</t>
   </si>
   <si>
     <t xml:space="preserve">Ladrillo KK 18 huecos (+5%)</t>
@@ -892,13 +895,13 @@
     <t xml:space="preserve">Eliminación de desmonte - volquete 18 m³</t>
   </si>
   <si>
-    <t xml:space="preserve">79.5 m³ suelto ÷ 18</t>
+    <t xml:space="preserve">81.7 m³ suelto ÷ 18</t>
   </si>
   <si>
     <t xml:space="preserve">Alquiler de apisonador para relleno</t>
   </si>
   <si>
-    <t xml:space="preserve">61 m³ ÷ 8 m³/día</t>
+    <t xml:space="preserve">59 m³ ÷ 8 m³/día</t>
   </si>
   <si>
     <t xml:space="preserve">1 por vaciado</t>
@@ -922,6 +925,12 @@
     <t xml:space="preserve">Precio por partida (destajo Lima). La excavación incluye la retroexcavadora y el carguío. Columnas H-J: uso interno (rendimiento de tu cuadrilla operario + ayudante).</t>
   </si>
   <si>
+    <t xml:space="preserve">Precio objetivo MO (S/)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factor</t>
+  </si>
+  <si>
     <t xml:space="preserve">Metrado</t>
   </si>
   <si>
@@ -934,6 +943,9 @@
     <t xml:space="preserve">Días-cuadrilla</t>
   </si>
   <si>
+    <t xml:space="preserve">P.U. base (S/)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Excavación con retroexcavadora (zapatas + zanjas) y carguío</t>
   </si>
   <si>
@@ -991,7 +1003,7 @@
     <t xml:space="preserve">Colocación de tecnopor bajo VE</t>
   </si>
   <si>
-    <t xml:space="preserve">Vaciado y vibrado premezclado - cimentación (40 m³)</t>
+    <t xml:space="preserve">Vaciado y vibrado premezclado - cimentación (42 m³)</t>
   </si>
   <si>
     <t xml:space="preserve">1 día + eventuales</t>
@@ -1051,7 +1063,7 @@
     <t xml:space="preserve">Limpieza final</t>
   </si>
   <si>
-    <t xml:space="preserve">Dirección técnica y residencia de obra (tú)</t>
+    <t xml:space="preserve">Dirección técnica y residencia de obra</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -1205,7 +1217,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -1213,9 +1225,10 @@
     <numFmt numFmtId="168" formatCode="\+#,##0.00;\-#,##0.00;\-"/>
     <numFmt numFmtId="169" formatCode="#,##0.0"/>
     <numFmt numFmtId="170" formatCode="0"/>
-    <numFmt numFmtId="171" formatCode="0.0"/>
-    <numFmt numFmtId="172" formatCode="#,##0"/>
-    <numFmt numFmtId="173" formatCode="0.00"/>
+    <numFmt numFmtId="171" formatCode="0.000"/>
+    <numFmt numFmtId="172" formatCode="0.0"/>
+    <numFmt numFmtId="173" formatCode="#,##0"/>
+    <numFmt numFmtId="174" formatCode="0.00"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -1394,7 +1407,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1499,11 +1512,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1511,7 +1532,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1519,19 +1552,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1826,11 +1847,11 @@
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">Materiales!$F$32</f>
-        <v>53330.89</v>
+        <v>54431.49</v>
       </c>
       <c r="C5" s="6" t="n">
         <f aca="false">B5/$B$10</f>
-        <v>0.580010255667419</v>
+        <v>0.554835612431767</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>7</v>
@@ -1846,7 +1867,7 @@
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">B6/$B$10</f>
-        <v>0.051278880878828</v>
+        <v>0.048061332008655</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>9</v>
@@ -1858,11 +1879,11 @@
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">'Mano de obra'!$F$34</f>
-        <v>31000</v>
+        <v>36000</v>
       </c>
       <c r="C7" s="6" t="n">
         <f aca="false">B7/$B$10</f>
-        <v>0.337146406626441</v>
+        <v>0.366958208337557</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>11</v>
@@ -1874,11 +1895,11 @@
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">SUM(B5:B7)</f>
-        <v>89045.89</v>
+        <v>95146.49</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">B8/$B$10</f>
-        <v>0.968435543172688</v>
+        <v>0.969855152777979</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1887,11 +1908,11 @@
       </c>
       <c r="B9" s="5" t="n">
         <f aca="false">0.05*(B5+B6)</f>
-        <v>2902.2945</v>
+        <v>2957.3245</v>
       </c>
       <c r="C9" s="6" t="n">
         <f aca="false">B9/$B$10</f>
-        <v>0.0315644568273123</v>
+        <v>0.0301448472220211</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>14</v>
@@ -1903,7 +1924,7 @@
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">B8+B9</f>
-        <v>91948.1845</v>
+        <v>98103.8145</v>
       </c>
       <c r="C10" s="6" t="n">
         <f aca="false">B10/$B$10</f>
@@ -1941,7 +1962,7 @@
       </c>
       <c r="B15" s="5" t="n">
         <f aca="false">$B$7*C15</f>
-        <v>4650</v>
+        <v>5400</v>
       </c>
       <c r="C15" s="10" t="n">
         <v>0.15</v>
@@ -1953,7 +1974,7 @@
       </c>
       <c r="B16" s="5" t="n">
         <f aca="false">$B$7*C16</f>
-        <v>9300</v>
+        <v>10800</v>
       </c>
       <c r="C16" s="10" t="n">
         <v>0.3</v>
@@ -1965,7 +1986,7 @@
       </c>
       <c r="B17" s="5" t="n">
         <f aca="false">$B$7*C17</f>
-        <v>3720</v>
+        <v>4320</v>
       </c>
       <c r="C17" s="10" t="n">
         <v>0.12</v>
@@ -1977,7 +1998,7 @@
       </c>
       <c r="B18" s="5" t="n">
         <f aca="false">$B$7*C18</f>
-        <v>7130</v>
+        <v>8280</v>
       </c>
       <c r="C18" s="10" t="n">
         <v>0.23</v>
@@ -1989,7 +2010,7 @@
       </c>
       <c r="B19" s="5" t="n">
         <f aca="false">$B$7*C19</f>
-        <v>6200</v>
+        <v>7200</v>
       </c>
       <c r="C19" s="10" t="n">
         <v>0.2</v>
@@ -2001,7 +2022,7 @@
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">SUM(B15:B19)</f>
-        <v>31000</v>
+        <v>36000</v>
       </c>
       <c r="C20" s="11" t="n">
         <f aca="false">SUM(C15:C19)</f>
@@ -2044,7 +2065,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -2244,11 +2265,11 @@
         <v>79.4</v>
       </c>
       <c r="E12" s="20" t="n">
-        <v>61.1</v>
+        <v>59.3</v>
       </c>
       <c r="F12" s="21" t="n">
         <f aca="false">E12-D12</f>
-        <v>-18.3</v>
+        <v>-20.1</v>
       </c>
       <c r="G12" s="22" t="s">
         <v>59</v>
@@ -2268,11 +2289,11 @@
         <v>53.5</v>
       </c>
       <c r="E13" s="20" t="n">
-        <v>79.5</v>
+        <v>81.7</v>
       </c>
       <c r="F13" s="21" t="n">
         <f aca="false">E13-D13</f>
-        <v>26</v>
+        <v>28.2</v>
       </c>
       <c r="G13" s="22" t="s">
         <v>62</v>
@@ -2337,51 +2358,51 @@
         <v>69</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+    <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="19" t="n">
         <v>2.7</v>
       </c>
-      <c r="E17" s="15" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="F17" s="16" t="n">
+      <c r="E17" s="20" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="F17" s="21" t="n">
         <f aca="false">E17-D17</f>
-        <v>0</v>
-      </c>
-      <c r="G17" s="17" t="s">
+        <v>1.59</v>
+      </c>
+      <c r="G17" s="22" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D18" s="19" t="n">
         <v>35.4</v>
       </c>
-      <c r="E18" s="15" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="F18" s="16" t="n">
+      <c r="E18" s="20" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="F18" s="21" t="n">
         <f aca="false">E18-D18</f>
-        <v>0</v>
-      </c>
-      <c r="G18" s="17" t="s">
+        <v>21.8</v>
+      </c>
+      <c r="G18" s="22" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2396,7 +2417,7 @@
       <c r="F19" s="14"/>
       <c r="G19" s="14"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
         <v>77</v>
       </c>
@@ -2833,6 +2854,11 @@
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="23" t="s">
         <v>133</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="23" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2863,37 +2889,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>49</v>
@@ -2902,15 +2928,15 @@
         <v>320</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>49</v>
@@ -2919,32 +2945,32 @@
         <v>38</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D7" s="15" t="n">
         <v>28.6</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>49</v>
@@ -2953,15 +2979,15 @@
         <v>65</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>49</v>
@@ -2970,15 +2996,15 @@
         <v>80</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>49</v>
@@ -2987,15 +3013,15 @@
         <v>60</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>49</v>
@@ -3004,15 +3030,15 @@
         <v>50</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>49</v>
@@ -3021,117 +3047,117 @@
         <v>50</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>80.02</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>164</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>163</v>
       </c>
       <c r="D14" s="15" t="n">
         <v>54.41</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D15" s="15" t="n">
         <v>35.96</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D16" s="15" t="n">
         <v>20.06</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D17" s="15" t="n">
         <v>7.96</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D18" s="15" t="n">
         <v>349.9</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>109</v>
@@ -3140,15 +3166,15 @@
         <v>6.5</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>109</v>
@@ -3157,15 +3183,15 @@
         <v>7.5</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>113</v>
@@ -3174,49 +3200,49 @@
         <v>1.14</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D22" s="15" t="n">
         <v>55</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>186</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>185</v>
       </c>
       <c r="D23" s="15" t="n">
         <v>16</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>113</v>
@@ -3225,66 +3251,66 @@
         <v>120</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D25" s="15" t="n">
         <v>45</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D26" s="15" t="n">
         <v>460</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D27" s="15" t="n">
         <v>130</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>130</v>
@@ -3293,49 +3319,49 @@
         <v>75</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D29" s="15" t="n">
         <v>20</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D30" s="15" t="n">
         <v>150</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>127</v>
@@ -3344,83 +3370,83 @@
         <v>300</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D32" s="15" t="n">
         <v>130</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D33" s="15" t="n">
         <v>80</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D34" s="15" t="n">
         <v>100</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D35" s="15" t="n">
         <v>80</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>113</v>
@@ -3429,15 +3455,15 @@
         <v>1000</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>113</v>
@@ -3446,32 +3472,32 @@
         <v>400</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D38" s="15" t="n">
         <v>95</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>113</v>
@@ -3480,15 +3506,15 @@
         <v>32</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>127</v>
@@ -3497,15 +3523,15 @@
         <v>900</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>4</v>
@@ -3514,7 +3540,7 @@
         <v>0.45</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -3546,40 +3572,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B5" s="14"/>
       <c r="C5" s="14"/>
@@ -3593,13 +3619,13 @@
         <v>1</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>49</v>
       </c>
       <c r="D6" s="24" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E6" s="5" t="n">
         <f aca="false">Precios!$D$5</f>
@@ -3607,10 +3633,10 @@
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">D6*E6</f>
-        <v>12800</v>
+        <v>13440</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3618,13 +3644,13 @@
         <v>2</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="24" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E7" s="5" t="n">
         <f aca="false">Precios!$D$6</f>
@@ -3632,7 +3658,7 @@
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">D7*E7</f>
-        <v>1520</v>
+        <v>1596</v>
       </c>
       <c r="G7" s="4"/>
     </row>
@@ -3641,7 +3667,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>49</v>
@@ -3658,7 +3684,7 @@
         <v>3040</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3666,7 +3692,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>49</v>
@@ -3683,12 +3709,12 @@
         <v>760</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
@@ -3702,13 +3728,13 @@
         <v>5</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D11" s="24" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="E11" s="5" t="n">
         <f aca="false">Precios!$D$7</f>
@@ -3716,10 +3742,10 @@
       </c>
       <c r="F11" s="5" t="n">
         <f aca="false">D11*E11</f>
-        <v>1744.6</v>
+        <v>1916.2</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3727,13 +3753,13 @@
         <v>6</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>49</v>
       </c>
       <c r="D12" s="24" t="n">
-        <v>9.6</v>
+        <v>11</v>
       </c>
       <c r="E12" s="5" t="n">
         <f aca="false">Precios!$D$10</f>
@@ -3741,10 +3767,10 @@
       </c>
       <c r="F12" s="5" t="n">
         <f aca="false">D12*E12</f>
-        <v>576</v>
+        <v>660</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3752,7 +3778,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>49</v>
@@ -3769,7 +3795,7 @@
         <v>195</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3777,7 +3803,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>49</v>
@@ -3800,7 +3826,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>49</v>
@@ -3823,13 +3849,13 @@
         <v>10</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>49</v>
       </c>
       <c r="D16" s="24" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="E16" s="5" t="n">
         <f aca="false">Precios!$D$12</f>
@@ -3837,13 +3863,13 @@
       </c>
       <c r="F16" s="5" t="n">
         <f aca="false">D16*E16</f>
-        <v>55</v>
+        <v>85</v>
       </c>
       <c r="G16" s="4"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
@@ -3857,10 +3883,10 @@
         <v>11</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D18" s="24" t="n">
         <v>72</v>
@@ -3874,7 +3900,7 @@
         <v>5761.44</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3882,10 +3908,10 @@
         <v>12</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D19" s="24" t="n">
         <v>207</v>
@@ -3899,7 +3925,7 @@
         <v>11262.87</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3907,10 +3933,10 @@
         <v>13</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D20" s="24" t="n">
         <v>179</v>
@@ -3924,7 +3950,7 @@
         <v>6436.84</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3932,10 +3958,10 @@
         <v>14</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D21" s="24" t="n">
         <v>134</v>
@@ -3949,7 +3975,7 @@
         <v>2688.04</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3957,10 +3983,10 @@
         <v>15</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D22" s="24" t="n">
         <v>15</v>
@@ -3974,7 +4000,7 @@
         <v>119.4</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3982,10 +4008,10 @@
         <v>16</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D23" s="24" t="n">
         <v>2</v>
@@ -3999,12 +4025,12 @@
         <v>699.8</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B24" s="14"/>
       <c r="C24" s="14"/>
@@ -4018,13 +4044,13 @@
         <v>17</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>109</v>
       </c>
       <c r="D25" s="24" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="E25" s="5" t="n">
         <f aca="false">Precios!$D$19</f>
@@ -4032,10 +4058,10 @@
       </c>
       <c r="F25" s="5" t="n">
         <f aca="false">D25*E25</f>
-        <v>364</v>
+        <v>403</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4043,13 +4069,13 @@
         <v>18</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>109</v>
       </c>
       <c r="D26" s="24" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E26" s="5" t="n">
         <f aca="false">Precios!$D$20</f>
@@ -4057,10 +4083,10 @@
       </c>
       <c r="F26" s="5" t="n">
         <f aca="false">D26*E26</f>
-        <v>262.5</v>
+        <v>277.5</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4068,7 +4094,7 @@
         <v>19</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>113</v>
@@ -4085,7 +4111,7 @@
         <v>4514.4</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4093,10 +4119,10 @@
         <v>20</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D28" s="24" t="n">
         <v>3</v>
@@ -4110,7 +4136,7 @@
         <v>165</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4118,10 +4144,10 @@
         <v>21</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D29" s="24" t="n">
         <v>5</v>
@@ -4135,7 +4161,7 @@
         <v>80</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4143,7 +4169,7 @@
         <v>22</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>113</v>
@@ -4160,7 +4186,7 @@
         <v>120</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4168,13 +4194,13 @@
         <v>23</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D31" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E31" s="5" t="n">
         <f aca="false">Precios!$D$25</f>
@@ -4182,7 +4208,7 @@
       </c>
       <c r="F31" s="5" t="n">
         <f aca="false">D31*E31</f>
-        <v>90</v>
+        <v>135</v>
       </c>
       <c r="G31" s="4"/>
     </row>
@@ -4192,7 +4218,7 @@
       </c>
       <c r="F32" s="8" t="n">
         <f aca="false">SUM(F5:F31)</f>
-        <v>53330.89</v>
+        <v>54431.49</v>
       </c>
     </row>
   </sheetData>
@@ -4225,7 +4251,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4233,7 +4259,7 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>2</v>
@@ -4242,16 +4268,16 @@
         <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4259,10 +4285,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D5" s="24" t="n">
         <v>5</v>
@@ -4276,7 +4302,7 @@
         <v>2300</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4284,10 +4310,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D6" s="24" t="n">
         <v>8</v>
@@ -4301,7 +4327,7 @@
         <v>1040</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4326,7 +4352,7 @@
         <v>375</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4334,10 +4360,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D8" s="24" t="n">
         <v>20</v>
@@ -4357,7 +4383,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>127</v>
@@ -4379,7 +4405,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>127</v>
@@ -4395,7 +4421,7 @@
         <v>300</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4423,7 +4449,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -4435,16 +4461,36 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="M3" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="N3" s="26" t="n">
+        <v>36000</v>
+      </c>
+      <c r="O3" s="9" t="s">
+        <v>300</v>
+      </c>
+      <c r="P3" s="27" t="n">
+        <f aca="false">N3/SUMPRODUCT(D5:D32,K5:K32)</f>
+        <v>1.14815322742683</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4458,23 +4504,26 @@
         <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4491,21 +4540,25 @@
         <f aca="false">Metrados!$E$6</f>
         <v>170</v>
       </c>
-      <c r="E5" s="15" t="n">
-        <v>2</v>
+      <c r="E5" s="5" t="n">
+        <f aca="false">ROUND(K5*$P$3,2)</f>
+        <v>2.3</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">D5*E5</f>
-        <v>340</v>
+        <v>391</v>
       </c>
       <c r="H5" s="24" t="n">
         <v>170</v>
       </c>
-      <c r="I5" s="26" t="n">
+      <c r="I5" s="28" t="n">
         <f aca="false">D5/H5</f>
         <v>1</v>
       </c>
       <c r="J5" s="4"/>
+      <c r="K5" s="15" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
@@ -4521,28 +4574,32 @@
         <f aca="false">Metrados!$E$7</f>
         <v>170</v>
       </c>
-      <c r="E6" s="15" t="n">
-        <v>3</v>
+      <c r="E6" s="5" t="n">
+        <f aca="false">ROUND(K6*$P$3,2)</f>
+        <v>3.44</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">D6*E6</f>
-        <v>510</v>
+        <v>584.8</v>
       </c>
       <c r="H6" s="24" t="n">
         <v>170</v>
       </c>
-      <c r="I6" s="26" t="n">
+      <c r="I6" s="28" t="n">
         <f aca="false">D6/H6</f>
         <v>1</v>
       </c>
       <c r="J6" s="4"/>
+      <c r="K6" s="15" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
         <v>47</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>49</v>
@@ -4551,21 +4608,25 @@
         <f aca="false">Metrados!$E$9+Metrados!$E$10</f>
         <v>111.4</v>
       </c>
-      <c r="E7" s="15" t="n">
-        <v>32</v>
+      <c r="E7" s="5" t="n">
+        <f aca="false">ROUND(K7*$P$3,2)</f>
+        <v>36.74</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">D7*E7</f>
-        <v>3564.8</v>
+        <v>4092.836</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="I7" s="26" t="n">
+        <v>307</v>
+      </c>
+      <c r="I7" s="28" t="n">
         <v>0</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>304</v>
+        <v>308</v>
+      </c>
+      <c r="K7" s="15" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4573,7 +4634,7 @@
         <v>51</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>42</v>
@@ -4581,22 +4642,26 @@
       <c r="D8" s="15" t="n">
         <v>75.2</v>
       </c>
-      <c r="E8" s="15" t="n">
-        <v>6</v>
+      <c r="E8" s="5" t="n">
+        <f aca="false">ROUND(K8*$P$3,2)</f>
+        <v>6.89</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">D8*E8</f>
-        <v>451.2</v>
+        <v>518.128</v>
       </c>
       <c r="H8" s="24" t="n">
         <v>25</v>
       </c>
-      <c r="I8" s="26" t="n">
+      <c r="I8" s="28" t="n">
         <f aca="false">D8/H8</f>
         <v>3.008</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>306</v>
+        <v>310</v>
+      </c>
+      <c r="K8" s="15" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4604,7 +4669,7 @@
         <v>54</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>49</v>
@@ -4613,52 +4678,60 @@
         <f aca="false">Metrados!$E$11</f>
         <v>13.3</v>
       </c>
-      <c r="E9" s="15" t="n">
-        <v>45</v>
+      <c r="E9" s="5" t="n">
+        <f aca="false">ROUND(K9*$P$3,2)</f>
+        <v>51.67</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">D9*E9</f>
-        <v>598.5</v>
+        <v>687.211</v>
       </c>
       <c r="H9" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="I9" s="26" t="n">
+      <c r="I9" s="28" t="n">
         <f aca="false">D9/H9</f>
         <v>3.325</v>
       </c>
       <c r="J9" s="4"/>
+      <c r="K9" s="15" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
         <v>57</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>49</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">Metrados!$E$12</f>
-        <v>61.1</v>
-      </c>
-      <c r="E10" s="15" t="n">
-        <v>30</v>
+        <v>59.3</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <f aca="false">ROUND(K10*$P$3,2)</f>
+        <v>34.44</v>
       </c>
       <c r="F10" s="5" t="n">
         <f aca="false">D10*E10</f>
-        <v>1833</v>
+        <v>2042.292</v>
       </c>
       <c r="H10" s="24" t="n">
         <v>8</v>
       </c>
-      <c r="I10" s="26" t="n">
+      <c r="I10" s="28" t="n">
         <f aca="false">D10/H10</f>
-        <v>7.6375</v>
+        <v>7.4125</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>309</v>
+        <v>313</v>
+      </c>
+      <c r="K10" s="15" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4666,7 +4739,7 @@
         <v>64</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>42</v>
@@ -4675,28 +4748,32 @@
         <f aca="false">Metrados!$E$15</f>
         <v>50</v>
       </c>
-      <c r="E11" s="15" t="n">
-        <v>15</v>
+      <c r="E11" s="5" t="n">
+        <f aca="false">ROUND(K11*$P$3,2)</f>
+        <v>17.22</v>
       </c>
       <c r="F11" s="5" t="n">
         <f aca="false">D11*E11</f>
-        <v>750</v>
+        <v>861</v>
       </c>
       <c r="H11" s="24" t="n">
         <v>35</v>
       </c>
-      <c r="I11" s="26" t="n">
+      <c r="I11" s="28" t="n">
         <f aca="false">D11/H11</f>
         <v>1.42857142857143</v>
       </c>
       <c r="J11" s="4"/>
+      <c r="K11" s="15" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
         <v>67</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>49</v>
@@ -4705,88 +4782,100 @@
         <f aca="false">Metrados!$E$16</f>
         <v>2.2</v>
       </c>
-      <c r="E12" s="15" t="n">
-        <v>90</v>
+      <c r="E12" s="5" t="n">
+        <f aca="false">ROUND(K12*$P$3,2)</f>
+        <v>103.33</v>
       </c>
       <c r="F12" s="5" t="n">
         <f aca="false">D12*E12</f>
-        <v>198</v>
+        <v>227.326</v>
       </c>
       <c r="H12" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="I12" s="26" t="n">
+      <c r="I12" s="28" t="n">
         <f aca="false">D12/H12</f>
         <v>0.55</v>
       </c>
       <c r="J12" s="4"/>
+      <c r="K12" s="15" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
         <v>70</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>49</v>
       </c>
       <c r="D13" s="5" t="n">
         <f aca="false">Metrados!$E$17</f>
-        <v>2.7</v>
-      </c>
-      <c r="E13" s="15" t="n">
-        <v>120</v>
+        <v>4.29</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <f aca="false">ROUND(K13*$P$3,2)</f>
+        <v>137.78</v>
       </c>
       <c r="F13" s="5" t="n">
         <f aca="false">D13*E13</f>
-        <v>324</v>
+        <v>591.0762</v>
       </c>
       <c r="H13" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="I13" s="26" t="n">
+      <c r="I13" s="28" t="n">
         <f aca="false">D13/H13</f>
-        <v>0.9</v>
+        <v>1.43</v>
       </c>
       <c r="J13" s="4"/>
+      <c r="K13" s="15" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
         <v>73</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>42</v>
       </c>
       <c r="D14" s="5" t="n">
         <f aca="false">Metrados!$E$18</f>
-        <v>35.4</v>
-      </c>
-      <c r="E14" s="15" t="n">
-        <v>22</v>
+        <v>57.2</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <f aca="false">ROUND(K14*$P$3,2)</f>
+        <v>25.26</v>
       </c>
       <c r="F14" s="5" t="n">
         <f aca="false">D14*E14</f>
-        <v>778.8</v>
+        <v>1444.872</v>
       </c>
       <c r="H14" s="24" t="n">
         <v>14</v>
       </c>
-      <c r="I14" s="26" t="n">
+      <c r="I14" s="28" t="n">
         <f aca="false">D14/H14</f>
-        <v>2.52857142857143</v>
+        <v>4.08571428571429</v>
       </c>
       <c r="J14" s="4"/>
+      <c r="K14" s="15" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>109</v>
@@ -4794,28 +4883,32 @@
       <c r="D15" s="15" t="n">
         <v>823</v>
       </c>
-      <c r="E15" s="15" t="n">
-        <v>1.1</v>
+      <c r="E15" s="5" t="n">
+        <f aca="false">ROUND(K15*$P$3,2)</f>
+        <v>1.26</v>
       </c>
       <c r="F15" s="5" t="n">
         <f aca="false">D15*E15</f>
-        <v>905.3</v>
+        <v>1036.98</v>
       </c>
       <c r="H15" s="24" t="n">
         <v>350</v>
       </c>
-      <c r="I15" s="26" t="n">
+      <c r="I15" s="28" t="n">
         <f aca="false">D15/H15</f>
         <v>2.35142857142857</v>
       </c>
       <c r="J15" s="4"/>
+      <c r="K15" s="15" t="n">
+        <v>1.1</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>109</v>
@@ -4823,28 +4916,32 @@
       <c r="D16" s="15" t="n">
         <v>2097</v>
       </c>
-      <c r="E16" s="15" t="n">
-        <v>1.1</v>
+      <c r="E16" s="5" t="n">
+        <f aca="false">ROUND(K16*$P$3,2)</f>
+        <v>1.26</v>
       </c>
       <c r="F16" s="5" t="n">
         <f aca="false">D16*E16</f>
-        <v>2306.7</v>
+        <v>2642.22</v>
       </c>
       <c r="H16" s="24" t="n">
         <v>250</v>
       </c>
-      <c r="I16" s="26" t="n">
+      <c r="I16" s="28" t="n">
         <f aca="false">D16/H16</f>
         <v>8.388</v>
       </c>
       <c r="J16" s="4"/>
+      <c r="K16" s="15" t="n">
+        <v>1.1</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
         <v>83</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>42</v>
@@ -4852,22 +4949,26 @@
       <c r="D17" s="15" t="n">
         <v>82.9</v>
       </c>
-      <c r="E17" s="15" t="n">
-        <v>25</v>
+      <c r="E17" s="5" t="n">
+        <f aca="false">ROUND(K17*$P$3,2)</f>
+        <v>28.7</v>
       </c>
       <c r="F17" s="5" t="n">
         <f aca="false">D17*E17</f>
-        <v>2072.5</v>
+        <v>2379.23</v>
       </c>
       <c r="H17" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="I17" s="26" t="n">
+      <c r="I17" s="28" t="n">
         <f aca="false">D17/H17</f>
         <v>6.90833333333333</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>319</v>
+        <v>323</v>
+      </c>
+      <c r="K17" s="15" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4875,7 +4976,7 @@
         <v>86</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>42</v>
@@ -4884,28 +4985,32 @@
         <f aca="false">Metrados!$E$23</f>
         <v>7.4</v>
       </c>
-      <c r="E18" s="15" t="n">
-        <v>5</v>
+      <c r="E18" s="5" t="n">
+        <f aca="false">ROUND(K18*$P$3,2)</f>
+        <v>5.74</v>
       </c>
       <c r="F18" s="5" t="n">
         <f aca="false">D18*E18</f>
-        <v>37</v>
+        <v>42.476</v>
       </c>
       <c r="H18" s="24" t="n">
         <v>50</v>
       </c>
-      <c r="I18" s="26" t="n">
+      <c r="I18" s="28" t="n">
         <f aca="false">D18/H18</f>
         <v>0.148</v>
       </c>
       <c r="J18" s="4"/>
+      <c r="K18" s="15" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
         <v>77</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>49</v>
@@ -4913,30 +5018,34 @@
       <c r="D19" s="15" t="n">
         <v>38.2</v>
       </c>
-      <c r="E19" s="15" t="n">
-        <v>40</v>
+      <c r="E19" s="5" t="n">
+        <f aca="false">ROUND(K19*$P$3,2)</f>
+        <v>45.93</v>
       </c>
       <c r="F19" s="5" t="n">
         <f aca="false">D19*E19</f>
-        <v>1528</v>
+        <v>1754.526</v>
       </c>
       <c r="H19" s="24" t="n">
         <v>38.2</v>
       </c>
-      <c r="I19" s="26" t="n">
+      <c r="I19" s="28" t="n">
         <f aca="false">D19/H19</f>
         <v>1</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>322</v>
+        <v>326</v>
+      </c>
+      <c r="K19" s="15" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>109</v>
@@ -4944,22 +5053,26 @@
       <c r="D20" s="15" t="n">
         <v>2646</v>
       </c>
-      <c r="E20" s="15" t="n">
-        <v>1.3</v>
+      <c r="E20" s="5" t="n">
+        <f aca="false">ROUND(K20*$P$3,2)</f>
+        <v>1.49</v>
       </c>
       <c r="F20" s="5" t="n">
         <f aca="false">D20*E20</f>
-        <v>3439.8</v>
+        <v>3942.54</v>
       </c>
       <c r="H20" s="24" t="n">
         <v>200</v>
       </c>
-      <c r="I20" s="26" t="n">
+      <c r="I20" s="28" t="n">
         <f aca="false">D20/H20</f>
         <v>13.23</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>325</v>
+        <v>329</v>
+      </c>
+      <c r="K20" s="15" t="n">
+        <v>1.3</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4967,7 +5080,7 @@
         <v>98</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>42</v>
@@ -4976,28 +5089,32 @@
         <f aca="false">Metrados!$E$27</f>
         <v>83.5</v>
       </c>
-      <c r="E21" s="15" t="n">
-        <v>28</v>
+      <c r="E21" s="5" t="n">
+        <f aca="false">ROUND(K21*$P$3,2)</f>
+        <v>32.15</v>
       </c>
       <c r="F21" s="5" t="n">
         <f aca="false">D21*E21</f>
-        <v>2338</v>
+        <v>2684.525</v>
       </c>
       <c r="H21" s="24" t="n">
         <v>10</v>
       </c>
-      <c r="I21" s="26" t="n">
+      <c r="I21" s="28" t="n">
         <f aca="false">D21/H21</f>
         <v>8.35</v>
       </c>
       <c r="J21" s="4"/>
+      <c r="K21" s="15" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
         <v>95</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>49</v>
@@ -5005,30 +5122,34 @@
       <c r="D22" s="15" t="n">
         <v>8.8</v>
       </c>
-      <c r="E22" s="15" t="n">
-        <v>60</v>
+      <c r="E22" s="5" t="n">
+        <f aca="false">ROUND(K22*$P$3,2)</f>
+        <v>68.89</v>
       </c>
       <c r="F22" s="5" t="n">
         <f aca="false">D22*E22</f>
-        <v>528</v>
+        <v>606.232</v>
       </c>
       <c r="H22" s="24" t="n">
         <v>8.8</v>
       </c>
-      <c r="I22" s="26" t="n">
+      <c r="I22" s="28" t="n">
         <f aca="false">D22/H22</f>
         <v>1</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>328</v>
+        <v>332</v>
+      </c>
+      <c r="K22" s="15" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>109</v>
@@ -5036,28 +5157,32 @@
       <c r="D23" s="15" t="n">
         <v>304</v>
       </c>
-      <c r="E23" s="15" t="n">
-        <v>1.2</v>
+      <c r="E23" s="5" t="n">
+        <f aca="false">ROUND(K23*$P$3,2)</f>
+        <v>1.38</v>
       </c>
       <c r="F23" s="5" t="n">
         <f aca="false">D23*E23</f>
-        <v>364.8</v>
+        <v>419.52</v>
       </c>
       <c r="H23" s="24" t="n">
         <v>150</v>
       </c>
-      <c r="I23" s="26" t="n">
+      <c r="I23" s="28" t="n">
         <f aca="false">D23/H23</f>
         <v>2.02666666666667</v>
       </c>
       <c r="J23" s="4"/>
+      <c r="K23" s="15" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
         <v>104</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>42</v>
@@ -5066,28 +5191,32 @@
         <f aca="false">Metrados!$E$29</f>
         <v>21.9</v>
       </c>
-      <c r="E24" s="15" t="n">
-        <v>25</v>
+      <c r="E24" s="5" t="n">
+        <f aca="false">ROUND(K24*$P$3,2)</f>
+        <v>28.7</v>
       </c>
       <c r="F24" s="5" t="n">
         <f aca="false">D24*E24</f>
-        <v>547.5</v>
+        <v>628.53</v>
       </c>
       <c r="H24" s="24" t="n">
         <v>10</v>
       </c>
-      <c r="I24" s="26" t="n">
+      <c r="I24" s="28" t="n">
         <f aca="false">D24/H24</f>
         <v>2.19</v>
       </c>
       <c r="J24" s="4"/>
+      <c r="K24" s="15" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>49</v>
@@ -5095,28 +5224,32 @@
       <c r="D25" s="15" t="n">
         <v>0.37</v>
       </c>
-      <c r="E25" s="15" t="n">
-        <v>120</v>
+      <c r="E25" s="5" t="n">
+        <f aca="false">ROUND(K25*$P$3,2)</f>
+        <v>137.78</v>
       </c>
       <c r="F25" s="5" t="n">
         <f aca="false">D25*E25</f>
-        <v>44.4</v>
+        <v>50.9786</v>
       </c>
       <c r="H25" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="I25" s="26" t="n">
+      <c r="I25" s="28" t="n">
         <f aca="false">D25/H25</f>
         <v>0.185</v>
       </c>
       <c r="J25" s="4"/>
+      <c r="K25" s="15" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
         <v>111</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>113</v>
@@ -5125,28 +5258,32 @@
         <f aca="false">Metrados!$E$31</f>
         <v>8</v>
       </c>
-      <c r="E26" s="15" t="n">
-        <v>20</v>
+      <c r="E26" s="5" t="n">
+        <f aca="false">ROUND(K26*$P$3,2)</f>
+        <v>22.96</v>
       </c>
       <c r="F26" s="5" t="n">
         <f aca="false">D26*E26</f>
-        <v>160</v>
+        <v>183.68</v>
       </c>
       <c r="H26" s="24" t="n">
         <v>16</v>
       </c>
-      <c r="I26" s="26" t="n">
+      <c r="I26" s="28" t="n">
         <f aca="false">D26/H26</f>
         <v>0.5</v>
       </c>
       <c r="J26" s="4"/>
+      <c r="K26" s="15" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
         <v>115</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>42</v>
@@ -5155,28 +5292,32 @@
         <f aca="false">Metrados!$E$33</f>
         <v>29.8</v>
       </c>
-      <c r="E27" s="15" t="n">
-        <v>35</v>
+      <c r="E27" s="5" t="n">
+        <f aca="false">ROUND(K27*$P$3,2)</f>
+        <v>40.19</v>
       </c>
       <c r="F27" s="5" t="n">
         <f aca="false">D27*E27</f>
-        <v>1043</v>
+        <v>1197.662</v>
       </c>
       <c r="H27" s="24" t="n">
         <v>10</v>
       </c>
-      <c r="I27" s="26" t="n">
+      <c r="I27" s="28" t="n">
         <f aca="false">D27/H27</f>
         <v>2.98</v>
       </c>
       <c r="J27" s="4"/>
+      <c r="K27" s="15" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
         <v>117</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>42</v>
@@ -5185,21 +5326,25 @@
         <f aca="false">Metrados!$E$34</f>
         <v>66.6</v>
       </c>
-      <c r="E28" s="15" t="n">
-        <v>35</v>
+      <c r="E28" s="5" t="n">
+        <f aca="false">ROUND(K28*$P$3,2)</f>
+        <v>40.19</v>
       </c>
       <c r="F28" s="5" t="n">
         <f aca="false">D28*E28</f>
-        <v>2331</v>
+        <v>2676.654</v>
       </c>
       <c r="H28" s="24" t="n">
         <v>10</v>
       </c>
-      <c r="I28" s="26" t="n">
+      <c r="I28" s="28" t="n">
         <f aca="false">D28/H28</f>
         <v>6.66</v>
       </c>
       <c r="J28" s="4"/>
+      <c r="K28" s="15" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
@@ -5215,59 +5360,67 @@
         <f aca="false">Metrados!$E$35</f>
         <v>48</v>
       </c>
-      <c r="E29" s="15" t="n">
-        <v>8</v>
+      <c r="E29" s="5" t="n">
+        <f aca="false">ROUND(K29*$P$3,2)</f>
+        <v>9.19</v>
       </c>
       <c r="F29" s="5" t="n">
         <f aca="false">D29*E29</f>
-        <v>384</v>
+        <v>441.12</v>
       </c>
       <c r="H29" s="24" t="n">
         <v>60</v>
       </c>
-      <c r="I29" s="26" t="n">
+      <c r="I29" s="28" t="n">
         <f aca="false">D29/H29</f>
         <v>0.8</v>
       </c>
       <c r="J29" s="4"/>
+      <c r="K29" s="15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
         <v>125</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D30" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="E30" s="15" t="n">
-        <v>40</v>
+      <c r="E30" s="5" t="n">
+        <f aca="false">ROUND(K30*$P$3,2)</f>
+        <v>45.93</v>
       </c>
       <c r="F30" s="5" t="n">
         <f aca="false">D30*E30</f>
-        <v>560</v>
+        <v>643.02</v>
       </c>
       <c r="H30" s="24" t="n">
         <v>14</v>
       </c>
-      <c r="I30" s="26" t="n">
+      <c r="I30" s="28" t="n">
         <f aca="false">D30/H30</f>
         <v>1</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>338</v>
+        <v>342</v>
+      </c>
+      <c r="K30" s="15" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>127</v>
@@ -5275,25 +5428,29 @@
       <c r="D31" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="15" t="n">
-        <v>300</v>
+      <c r="E31" s="5" t="n">
+        <f aca="false">ROUND(K31*$P$3,2)</f>
+        <v>344.45</v>
       </c>
       <c r="F31" s="5" t="n">
         <f aca="false">D31*E31</f>
-        <v>300</v>
+        <v>344.45</v>
       </c>
       <c r="H31" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="I31" s="26" t="n">
+      <c r="I31" s="28" t="n">
         <f aca="false">D31/H31</f>
         <v>1</v>
       </c>
       <c r="J31" s="4"/>
+      <c r="K31" s="15" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="4" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>127</v>
@@ -5301,11 +5458,15 @@
       <c r="D32" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="15" t="n">
-        <v>2500</v>
+      <c r="E32" s="5" t="n">
+        <f aca="false">ROUND(K32*$P$3,2)</f>
+        <v>2870.38</v>
       </c>
       <c r="F32" s="5" t="n">
         <f aca="false">D32*E32</f>
+        <v>2870.38</v>
+      </c>
+      <c r="K32" s="15" t="n">
         <v>2500</v>
       </c>
     </row>
@@ -5315,23 +5476,23 @@
       </c>
       <c r="F33" s="8" t="n">
         <f aca="false">SUM(F5:F32)</f>
-        <v>30738.3</v>
+        <v>35985.2648</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>342</v>
-      </c>
-      <c r="I33" s="27" t="n">
+        <v>346</v>
+      </c>
+      <c r="I33" s="29" t="n">
         <f aca="false">SUM(I5:I31)</f>
-        <v>80.0950714285714</v>
+        <v>81.9572142857143</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E34" s="28" t="s">
-        <v>343</v>
-      </c>
-      <c r="F34" s="29" t="n">
-        <f aca="false">CEILING(F33,500)</f>
-        <v>31000</v>
+      <c r="E34" s="30" t="s">
+        <v>347</v>
+      </c>
+      <c r="F34" s="31" t="n">
+        <f aca="false">ROUND(F33,-2)</f>
+        <v>36000</v>
       </c>
     </row>
   </sheetData>
@@ -5360,12 +5521,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5373,68 +5534,68 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>348</v>
-      </c>
-      <c r="B5" s="26" t="n">
+        <v>352</v>
+      </c>
+      <c r="B5" s="28" t="n">
         <f aca="false">'Mano de obra'!$I$33</f>
-        <v>80.0950714285714</v>
+        <v>81.9572142857143</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>350</v>
-      </c>
-      <c r="B6" s="30" t="n">
+        <v>354</v>
+      </c>
+      <c r="B6" s="32" t="n">
         <v>1.35</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="B7" s="31" t="n">
+        <v>356</v>
+      </c>
+      <c r="B7" s="33" t="n">
         <v>0.1</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>354</v>
-      </c>
-      <c r="B8" s="32" t="n">
+        <v>358</v>
+      </c>
+      <c r="B8" s="34" t="n">
         <f aca="false">ROUNDUP(B5/B6*(1+B7),0)</f>
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="B9" s="26" t="n">
+        <v>360</v>
+      </c>
+      <c r="B9" s="28" t="n">
         <f aca="false">B8/6</f>
-        <v>11</v>
+        <v>11.1666666666667</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5442,108 +5603,108 @@
       <c r="C10" s="4"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
-        <v>358</v>
+      <c r="A11" s="30" t="s">
+        <v>362</v>
       </c>
       <c r="C11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>359</v>
-      </c>
-      <c r="B12" s="32" t="n">
+        <v>363</v>
+      </c>
+      <c r="B12" s="34" t="n">
         <f aca="false">B8*Precios!$D$32</f>
-        <v>8580</v>
+        <v>8710</v>
       </c>
       <c r="C12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>360</v>
-      </c>
-      <c r="B13" s="32" t="n">
+        <v>364</v>
+      </c>
+      <c r="B13" s="34" t="n">
         <f aca="false">B8*Precios!$D$33</f>
-        <v>5280</v>
+        <v>5360</v>
       </c>
       <c r="C13" s="4"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>361</v>
-      </c>
-      <c r="B14" s="32" t="n">
+        <v>365</v>
+      </c>
+      <c r="B14" s="34" t="n">
         <f aca="false">6*Precios!$D$33</f>
         <v>480</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>363</v>
-      </c>
-      <c r="B15" s="32" t="n">
+        <v>367</v>
+      </c>
+      <c r="B15" s="34" t="n">
         <f aca="false">13*Precios!$D$30</f>
         <v>1950</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="B16" s="32" t="n">
+        <v>210</v>
+      </c>
+      <c r="B16" s="34" t="n">
         <f aca="false">Precios!$D$31</f>
         <v>300</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>366</v>
-      </c>
-      <c r="B17" s="32" t="n">
+        <v>370</v>
+      </c>
+      <c r="B17" s="34" t="n">
         <f aca="false">Precios!$D$36</f>
         <v>1000</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>368</v>
-      </c>
-      <c r="B18" s="32" t="n">
+        <v>372</v>
+      </c>
+      <c r="B18" s="34" t="n">
         <f aca="false">Precios!$D$37</f>
         <v>400</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>369</v>
-      </c>
-      <c r="B19" s="32" t="n">
+        <v>373</v>
+      </c>
+      <c r="B19" s="34" t="n">
         <f aca="false">Precios!$D$39*Precios!$D$38</f>
         <v>3040</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>371</v>
-      </c>
-      <c r="B20" s="32" t="n">
+        <v>375</v>
+      </c>
+      <c r="B20" s="34" t="n">
         <f aca="false">Precios!$D$40</f>
         <v>900</v>
       </c>
@@ -5551,42 +5712,42 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>372</v>
-      </c>
-      <c r="B21" s="33" t="n">
+        <v>376</v>
+      </c>
+      <c r="B21" s="35" t="n">
         <v>600</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>374</v>
-      </c>
-      <c r="B22" s="33" t="n">
+        <v>378</v>
+      </c>
+      <c r="B22" s="35" t="n">
         <v>400</v>
       </c>
       <c r="C22" s="4"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>375</v>
-      </c>
-      <c r="B23" s="33" t="n">
+        <v>379</v>
+      </c>
+      <c r="B23" s="35" t="n">
         <v>600</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>377</v>
-      </c>
-      <c r="B24" s="34" t="n">
+        <v>381</v>
+      </c>
+      <c r="B24" s="36" t="n">
         <f aca="false">SUM(B12:B23)</f>
-        <v>23530</v>
+        <v>23740</v>
       </c>
       <c r="C24" s="4"/>
     </row>
@@ -5596,95 +5757,95 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>378</v>
-      </c>
-      <c r="B26" s="34" t="n">
+        <v>382</v>
+      </c>
+      <c r="B26" s="36" t="n">
         <f aca="false">'Mano de obra'!$F$34</f>
-        <v>31000</v>
+        <v>36000</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>380</v>
-      </c>
-      <c r="B27" s="34" t="n">
+        <v>384</v>
+      </c>
+      <c r="B27" s="36" t="n">
         <f aca="false">B26-B24</f>
-        <v>7470</v>
+        <v>12260</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>382</v>
-      </c>
-      <c r="B28" s="32" t="n">
+        <v>386</v>
+      </c>
+      <c r="B28" s="34" t="n">
         <f aca="false">(B17+B18+B19+B20)*Precios!$D$41</f>
         <v>2403</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>384</v>
-      </c>
-      <c r="B29" s="34" t="n">
+        <v>388</v>
+      </c>
+      <c r="B29" s="36" t="n">
         <f aca="false">B27+B28</f>
-        <v>9873</v>
+        <v>14663</v>
       </c>
       <c r="C29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>385</v>
-      </c>
-      <c r="B30" s="32" t="n">
+        <v>389</v>
+      </c>
+      <c r="B30" s="34" t="n">
         <f aca="false">B29/B9</f>
-        <v>897.545454545455</v>
+        <v>1313.10447761194</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="B31" s="6" t="n">
         <f aca="false">B29/B26</f>
-        <v>0.318483870967742</v>
+        <v>0.407305555555556</v>
       </c>
       <c r="C31" s="4"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="25" t="n">
         <v>50</v>
       </c>
-      <c r="B35" s="32" t="n">
+      <c r="B35" s="34" t="n">
         <f aca="false">B29-(50-B8)*(Precios!$D$32+Precios!$D$33)</f>
-        <v>13233</v>
+        <v>18233</v>
       </c>
       <c r="C35" s="4"/>
     </row>
@@ -5692,9 +5853,9 @@
       <c r="A36" s="25" t="n">
         <v>60</v>
       </c>
-      <c r="B36" s="32" t="n">
+      <c r="B36" s="34" t="n">
         <f aca="false">B29-(60-B8)*(Precios!$D$32+Precios!$D$33)</f>
-        <v>11133</v>
+        <v>16133</v>
       </c>
       <c r="C36" s="4"/>
     </row>
@@ -5702,9 +5863,9 @@
       <c r="A37" s="25" t="n">
         <v>70</v>
       </c>
-      <c r="B37" s="32" t="n">
+      <c r="B37" s="34" t="n">
         <f aca="false">B29-(70-B8)*(Precios!$D$32+Precios!$D$33)</f>
-        <v>9033</v>
+        <v>14033</v>
       </c>
       <c r="C37" s="4"/>
     </row>
@@ -5712,9 +5873,9 @@
       <c r="A38" s="25" t="n">
         <v>80</v>
       </c>
-      <c r="B38" s="32" t="n">
+      <c r="B38" s="34" t="n">
         <f aca="false">B29-(80-B8)*(Precios!$D$32+Precios!$D$33)</f>
-        <v>6933</v>
+        <v>11933</v>
       </c>
       <c r="C38" s="4"/>
     </row>
@@ -5722,9 +5883,9 @@
       <c r="A39" s="25" t="n">
         <v>90</v>
       </c>
-      <c r="B39" s="32" t="n">
+      <c r="B39" s="34" t="n">
         <f aca="false">B29-(90-B8)*(Precios!$D$32+Precios!$D$33)</f>
-        <v>4833</v>
+        <v>9833</v>
       </c>
       <c r="C39" s="4"/>
     </row>

</xml_diff>